<commit_message>
swarm ex eow bookeeping
</commit_message>
<xml_diff>
--- a/SWARM-EX/Planning/COMMS - Personal Waterfall Chart Justin Le.xlsx
+++ b/SWARM-EX/Planning/COMMS - Personal Waterfall Chart Justin Le.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12210" tabRatio="500"/>
+    <workbookView windowWidth="28800" windowHeight="12300" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="89">
   <si>
     <t>Total Hours</t>
   </si>
@@ -304,22 +304,22 @@
     <t>MCT: Review test docs</t>
   </si>
   <si>
+    <t>MCT: Bench setup</t>
+  </si>
+  <si>
+    <t>Learning Hydra</t>
+  </si>
+  <si>
+    <t>MCT: Hydra development</t>
+  </si>
+  <si>
+    <t>MCT: Hydra hardwired to Li2</t>
+  </si>
+  <si>
+    <t>MCT: Hydra hardwired to CDH to Li2</t>
+  </si>
+  <si>
     <t>Late (In Progress)</t>
-  </si>
-  <si>
-    <t>MCT: Bench setup</t>
-  </si>
-  <si>
-    <t>Learning Hydra</t>
-  </si>
-  <si>
-    <t>MCT: Hydra development</t>
-  </si>
-  <si>
-    <t>MCT: Hydra hardwired to Li2</t>
-  </si>
-  <si>
-    <t>MCT: Hydra hardwired to CDH to Li2</t>
   </si>
   <si>
     <t>MCT: Practice run-through of test</t>
@@ -422,11 +422,11 @@
   <numFmts count="5">
     <numFmt numFmtId="176" formatCode="m\/d"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="34">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -523,13 +523,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="13"/>
       <color theme="3"/>
@@ -538,8 +531,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -552,10 +560,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -591,14 +600,6 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -623,7 +624,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -636,17 +637,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -657,18 +664,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="48">
@@ -770,7 +765,121 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -782,49 +891,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -836,121 +945,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1332,16 +1327,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
+      <right style="double">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top style="thin">
+      <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="thin">
+      <bottom style="double">
         <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
@@ -1356,16 +1351,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <left style="thin">
         <color rgb="FF3F3F3F"/>
       </left>
-      <right style="double">
+      <right style="thin">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top style="double">
+      <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
+      <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
@@ -1388,134 +1383,134 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="34" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="35" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="44" borderId="36" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="30" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="34" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="33" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="44" borderId="36" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="30" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="37" borderId="35" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="33" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2307,7 +2302,7 @@
       </c>
       <c r="E3" s="23">
         <f t="shared" ref="E3:E64" si="1">SUM(F3:W3)</f>
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F3" s="24">
         <f t="shared" ref="F3:V3" si="2">F4+F7+F11+F14</f>
@@ -2331,7 +2326,7 @@
       </c>
       <c r="K3" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L3" s="24">
         <f t="shared" si="2"/>
@@ -2400,7 +2395,7 @@
       </c>
       <c r="E4" s="25">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F4" s="26">
         <f t="shared" ref="F4:W4" si="3">SUM(F5:F6)</f>
@@ -2424,7 +2419,7 @@
       </c>
       <c r="K4" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L4" s="26">
         <f t="shared" si="3"/>
@@ -2499,7 +2494,7 @@
       </c>
       <c r="E5" s="25">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="27">
         <v>1</v>
@@ -2516,7 +2511,9 @@
       <c r="J5" s="26">
         <v>1</v>
       </c>
-      <c r="K5" s="26"/>
+      <c r="K5" s="26">
+        <v>1</v>
+      </c>
       <c r="L5" s="26"/>
       <c r="M5" s="26"/>
       <c r="N5" s="26"/>
@@ -2554,7 +2551,7 @@
       </c>
       <c r="E6" s="28">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F6" s="29">
         <v>2</v>
@@ -2571,7 +2568,9 @@
       <c r="J6" s="30">
         <v>2</v>
       </c>
-      <c r="K6" s="30"/>
+      <c r="K6" s="30">
+        <v>2</v>
+      </c>
       <c r="L6" s="30"/>
       <c r="M6" s="30"/>
       <c r="N6" s="30"/>
@@ -2608,7 +2607,7 @@
       </c>
       <c r="E7" s="25">
         <f t="shared" si="1"/>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F7" s="31">
         <f t="shared" ref="F7:W7" si="4">SUM(F8:F10)</f>
@@ -2632,7 +2631,7 @@
       </c>
       <c r="K7" s="31">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L7" s="31">
         <f t="shared" si="4"/>
@@ -2705,7 +2704,7 @@
       </c>
       <c r="E8" s="25">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="27">
         <v>1</v>
@@ -2722,7 +2721,9 @@
       <c r="J8" s="26">
         <v>1</v>
       </c>
-      <c r="K8" s="26"/>
+      <c r="K8" s="26">
+        <v>1</v>
+      </c>
       <c r="L8" s="26"/>
       <c r="M8" s="26"/>
       <c r="N8" s="26"/>
@@ -2758,7 +2759,7 @@
       </c>
       <c r="E9" s="25">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9" s="27">
         <v>1</v>
@@ -2775,7 +2776,9 @@
       <c r="J9" s="26">
         <v>1</v>
       </c>
-      <c r="K9" s="26"/>
+      <c r="K9" s="26">
+        <v>1</v>
+      </c>
       <c r="L9" s="26"/>
       <c r="M9" s="26"/>
       <c r="N9" s="26"/>
@@ -2807,7 +2810,7 @@
       </c>
       <c r="E10" s="28">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" s="29">
         <v>2</v>
@@ -2824,7 +2827,9 @@
       <c r="J10" s="30">
         <v>3</v>
       </c>
-      <c r="K10" s="30"/>
+      <c r="K10" s="30">
+        <v>2</v>
+      </c>
       <c r="L10" s="30"/>
       <c r="M10" s="30"/>
       <c r="N10" s="30"/>
@@ -3238,7 +3243,7 @@
       </c>
       <c r="E17" s="23">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F17" s="32">
         <f t="shared" ref="F17:V17" si="7">F18+F21+F23+F26</f>
@@ -3262,7 +3267,7 @@
       </c>
       <c r="K17" s="32">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="32">
         <f t="shared" si="7"/>
@@ -3509,7 +3514,7 @@
       </c>
       <c r="E21" s="25">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F21" s="31">
         <f t="shared" ref="F21:W21" si="9">SUM(F22)</f>
@@ -3533,7 +3538,7 @@
       </c>
       <c r="K21" s="31">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="31">
         <f t="shared" si="9"/>
@@ -3604,7 +3609,7 @@
       </c>
       <c r="E22" s="25">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" s="27"/>
       <c r="G22" s="26"/>
@@ -3617,7 +3622,9 @@
       <c r="J22" s="26">
         <v>1</v>
       </c>
-      <c r="K22" s="26"/>
+      <c r="K22" s="26">
+        <v>1</v>
+      </c>
       <c r="L22" s="26"/>
       <c r="M22" s="26"/>
       <c r="N22" s="26"/>
@@ -3931,7 +3938,7 @@
       </c>
       <c r="E29" s="23">
         <f t="shared" si="1"/>
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F29" s="32">
         <f t="shared" ref="F29:V29" si="12">F30+F40+F47+F52+F62</f>
@@ -3955,7 +3962,7 @@
       </c>
       <c r="K29" s="32">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="L29" s="32">
         <f t="shared" si="12"/>
@@ -4020,7 +4027,7 @@
       </c>
       <c r="E30" s="25">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F30" s="31">
         <f t="shared" ref="F30:W30" si="13">SUM(F31:F39)</f>
@@ -4044,7 +4051,7 @@
       </c>
       <c r="K30" s="34">
         <f t="shared" si="13"/>
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="L30" s="34">
         <f t="shared" si="13"/>
@@ -4140,7 +4147,7 @@
       <c r="V31" s="26"/>
       <c r="W31" s="26"/>
       <c r="X31" s="58" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="Y31" s="59"/>
       <c r="Z31" s="59"/>
@@ -4151,7 +4158,7 @@
       <c r="A32" s="9"/>
       <c r="B32" s="12"/>
       <c r="C32" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D32" s="11">
         <v>2</v>
@@ -4183,7 +4190,7 @@
       <c r="V32" s="26"/>
       <c r="W32" s="26"/>
       <c r="X32" s="58" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="Y32" s="59"/>
       <c r="Z32" s="59"/>
@@ -4194,7 +4201,7 @@
       <c r="A33" s="9"/>
       <c r="B33" s="12"/>
       <c r="C33" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D33" s="11">
         <v>4</v>
@@ -4223,7 +4230,9 @@
       <c r="U33" s="26"/>
       <c r="V33" s="26"/>
       <c r="W33" s="26"/>
-      <c r="X33" s="58"/>
+      <c r="X33" s="58" t="s">
+        <v>16</v>
+      </c>
       <c r="Y33" s="59"/>
       <c r="Z33" s="59"/>
       <c r="AA33" s="59"/>
@@ -4233,21 +4242,23 @@
       <c r="A34" s="9"/>
       <c r="B34" s="12"/>
       <c r="C34" s="13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D34" s="11">
         <v>4</v>
       </c>
       <c r="E34" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F34" s="27"/>
       <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="39"/>
       <c r="J34" s="26"/>
-      <c r="K34" s="40"/>
+      <c r="K34" s="40">
+        <v>4</v>
+      </c>
       <c r="L34" s="26"/>
       <c r="M34" s="26"/>
       <c r="N34" s="26"/>
@@ -4260,7 +4271,9 @@
       <c r="U34" s="26"/>
       <c r="V34" s="26"/>
       <c r="W34" s="26"/>
-      <c r="X34" s="58"/>
+      <c r="X34" s="58" t="s">
+        <v>16</v>
+      </c>
       <c r="Y34" s="59"/>
       <c r="Z34" s="59"/>
       <c r="AA34" s="59"/>
@@ -4270,21 +4283,23 @@
       <c r="A35" s="9"/>
       <c r="B35" s="12"/>
       <c r="C35" s="13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D35" s="11">
         <v>4</v>
       </c>
       <c r="E35" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F35" s="27"/>
       <c r="G35" s="26"/>
       <c r="H35" s="26"/>
       <c r="I35" s="39"/>
       <c r="J35" s="26"/>
-      <c r="K35" s="40"/>
+      <c r="K35" s="40">
+        <v>4</v>
+      </c>
       <c r="L35" s="26"/>
       <c r="M35" s="26"/>
       <c r="N35" s="26"/>
@@ -4297,7 +4312,9 @@
       <c r="U35" s="26"/>
       <c r="V35" s="26"/>
       <c r="W35" s="26"/>
-      <c r="X35" s="58"/>
+      <c r="X35" s="58" t="s">
+        <v>16</v>
+      </c>
       <c r="Y35" s="59"/>
       <c r="Z35" s="59"/>
       <c r="AA35" s="59"/>
@@ -4307,21 +4324,23 @@
       <c r="A36" s="9"/>
       <c r="B36" s="12"/>
       <c r="C36" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D36" s="11">
         <v>4</v>
       </c>
       <c r="E36" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F36" s="27"/>
       <c r="G36" s="26"/>
       <c r="H36" s="26"/>
       <c r="I36" s="39"/>
       <c r="J36" s="26"/>
-      <c r="K36" s="40"/>
+      <c r="K36" s="40">
+        <v>2</v>
+      </c>
       <c r="L36" s="26"/>
       <c r="M36" s="26"/>
       <c r="N36" s="26"/>
@@ -4334,7 +4353,9 @@
       <c r="U36" s="26"/>
       <c r="V36" s="26"/>
       <c r="W36" s="26"/>
-      <c r="X36" s="58"/>
+      <c r="X36" s="58" t="s">
+        <v>57</v>
+      </c>
       <c r="Y36" s="59"/>
       <c r="Z36" s="59"/>
       <c r="AA36" s="59"/>
@@ -4351,14 +4372,16 @@
       </c>
       <c r="E37" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="27"/>
       <c r="G37" s="26"/>
       <c r="H37" s="26"/>
       <c r="I37" s="39"/>
       <c r="J37" s="26"/>
-      <c r="K37" s="40"/>
+      <c r="K37" s="40">
+        <v>1</v>
+      </c>
       <c r="L37" s="26"/>
       <c r="M37" s="26"/>
       <c r="N37" s="26"/>
@@ -4795,7 +4818,7 @@
       </c>
       <c r="E47" s="25">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F47" s="31">
         <f t="shared" ref="F47:W47" si="15">SUM(F48:F51)</f>
@@ -4819,7 +4842,7 @@
       </c>
       <c r="K47" s="34">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L47" s="34">
         <f t="shared" si="15"/>
@@ -5007,7 +5030,7 @@
       </c>
       <c r="E51" s="28">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F51" s="29"/>
       <c r="G51" s="30">
@@ -5018,7 +5041,9 @@
       </c>
       <c r="I51" s="30"/>
       <c r="J51" s="30"/>
-      <c r="K51" s="30"/>
+      <c r="K51" s="30">
+        <v>2</v>
+      </c>
       <c r="L51" s="30"/>
       <c r="M51" s="30"/>
       <c r="N51" s="41"/>
@@ -5673,7 +5698,7 @@
       </c>
       <c r="E65" s="83">
         <f t="shared" si="18"/>
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="F65" s="83">
         <f t="shared" si="18"/>
@@ -5697,7 +5722,7 @@
       </c>
       <c r="K65" s="83">
         <f t="shared" si="18"/>
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="L65" s="83">
         <f t="shared" si="18"/>
@@ -5828,7 +5853,7 @@
       </c>
       <c r="E67" s="84">
         <f t="shared" si="19"/>
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="F67" s="84">
         <f t="shared" si="19"/>
@@ -5852,7 +5877,7 @@
       </c>
       <c r="K67" s="84">
         <f t="shared" si="19"/>
-        <v>13</v>
+        <v>-8</v>
       </c>
       <c r="L67" s="84">
         <f t="shared" si="19"/>

</xml_diff>